<commit_message>
Fix MODE errors in Manual_Statistics sheet — use MODE.SNGL with IFERROR, add duplicate values to Sales_Data
</commit_message>
<xml_diff>
--- a/rFLA300/chapter-12/02_Descriptive_Statistics.xlsx
+++ b/rFLA300/chapter-12/02_Descriptive_Statistics.xlsx
@@ -19,10 +19,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="MMM DD, YYYY"/>
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="MMM DD, YYYY"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="MM/DD/YYYY"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -121,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -132,16 +132,73 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="167" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -150,44 +207,8 @@
     <xf numFmtId="166" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -614,687 +635,687 @@
       <c r="A3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="23" t="n">
         <v>45293</v>
       </c>
-      <c r="C3" s="5" t="n">
-        <v>8438</v>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>3445</v>
+      <c r="C3" s="24" t="n">
+        <v>8618</v>
+      </c>
+      <c r="D3" s="24" t="n">
+        <v>4804</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>141</v>
-      </c>
-      <c r="F3" s="6" t="n">
-        <v>89.54000000000001</v>
+        <v>158</v>
+      </c>
+      <c r="F3" s="25" t="n">
+        <v>67.27</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="26" t="n">
         <v>45294</v>
       </c>
-      <c r="C4" s="9" t="n">
-        <v>4112</v>
-      </c>
-      <c r="D4" s="9" t="n">
-        <v>7322</v>
+      <c r="C4" s="27" t="n">
+        <v>8238</v>
+      </c>
+      <c r="D4" s="27" t="n">
+        <v>5100</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>157</v>
-      </c>
-      <c r="F4" s="10" t="n">
-        <v>68.13</v>
+        <v>196</v>
+      </c>
+      <c r="F4" s="28" t="n">
+        <v>38.34</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="23" t="n">
         <v>45295</v>
       </c>
-      <c r="C5" s="5" t="n">
-        <v>3404</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>5201</v>
+      <c r="C5" s="24" t="n">
+        <v>4800</v>
+      </c>
+      <c r="D5" s="24" t="n">
+        <v>8865</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>76</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>60.74</v>
+        <v>155</v>
+      </c>
+      <c r="F5" s="25" t="n">
+        <v>94.95</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="26" t="n">
         <v>45296</v>
       </c>
-      <c r="C6" s="9" t="n">
-        <v>9274</v>
-      </c>
-      <c r="D6" s="9" t="n">
-        <v>7949</v>
+      <c r="C6" s="27" t="n">
+        <v>11821</v>
+      </c>
+      <c r="D6" s="27" t="n">
+        <v>3329</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>107</v>
-      </c>
-      <c r="F6" s="10" t="n">
-        <v>35.5</v>
+        <v>173</v>
+      </c>
+      <c r="F6" s="28" t="n">
+        <v>50.72</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="23" t="n">
         <v>45297</v>
       </c>
-      <c r="C7" s="5" t="n">
-        <v>5453</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>7866</v>
+      <c r="C7" s="24" t="n">
+        <v>4929</v>
+      </c>
+      <c r="D7" s="24" t="n">
+        <v>8970</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>75</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>52.32</v>
+        <v>139</v>
+      </c>
+      <c r="F7" s="25" t="n">
+        <v>39.52</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="26" t="n">
         <v>45298</v>
       </c>
-      <c r="C8" s="9" t="n">
-        <v>5206</v>
-      </c>
-      <c r="D8" s="9" t="n">
-        <v>5762</v>
+      <c r="C8" s="27" t="n">
+        <v>7200</v>
+      </c>
+      <c r="D8" s="27" t="n">
+        <v>3409</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>103</v>
-      </c>
-      <c r="F8" s="10" t="n">
-        <v>94.02</v>
+        <v>115</v>
+      </c>
+      <c r="F8" s="28" t="n">
+        <v>98.76000000000001</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="23" t="n">
         <v>45299</v>
       </c>
-      <c r="C9" s="5" t="n">
-        <v>5028</v>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>7529</v>
+      <c r="C9" s="24" t="n">
+        <v>6070</v>
+      </c>
+      <c r="D9" s="24" t="n">
+        <v>4341</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>183</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>82.05</v>
+        <v>158</v>
+      </c>
+      <c r="F9" s="25" t="n">
+        <v>56.67</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="26" t="n">
         <v>45300</v>
       </c>
-      <c r="C10" s="9" t="n">
-        <v>4343</v>
-      </c>
-      <c r="D10" s="9" t="n">
-        <v>4375</v>
+      <c r="C10" s="27" t="n">
+        <v>4183</v>
+      </c>
+      <c r="D10" s="27" t="n">
+        <v>6300</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>177</v>
-      </c>
-      <c r="F10" s="10" t="n">
-        <v>44.04</v>
+        <v>172</v>
+      </c>
+      <c r="F10" s="28" t="n">
+        <v>67.90000000000001</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B11" s="23" t="n">
         <v>45301</v>
       </c>
-      <c r="C11" s="5" t="n">
-        <v>9233</v>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>8571</v>
+      <c r="C11" s="24" t="n">
+        <v>3418</v>
+      </c>
+      <c r="D11" s="24" t="n">
+        <v>2092</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>107</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>44.14</v>
+        <v>77</v>
+      </c>
+      <c r="F11" s="25" t="n">
+        <v>75.28</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="26" t="n">
         <v>45302</v>
       </c>
-      <c r="C12" s="9" t="n">
-        <v>4039</v>
-      </c>
-      <c r="D12" s="9" t="n">
-        <v>3369</v>
+      <c r="C12" s="27" t="n">
+        <v>6114</v>
+      </c>
+      <c r="D12" s="27" t="n">
+        <v>8243</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>189</v>
-      </c>
-      <c r="F12" s="10" t="n">
-        <v>66.01000000000001</v>
+        <v>182</v>
+      </c>
+      <c r="F12" s="28" t="n">
+        <v>77.98999999999999</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="23" t="n">
         <v>45303</v>
       </c>
-      <c r="C13" s="5" t="n">
-        <v>8743</v>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>3175</v>
+      <c r="C13" s="24" t="n">
+        <v>9500</v>
+      </c>
+      <c r="D13" s="24" t="n">
+        <v>7401</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>149</v>
-      </c>
-      <c r="F13" s="6" t="n">
-        <v>33.28</v>
+        <v>170</v>
+      </c>
+      <c r="F13" s="25" t="n">
+        <v>109.34</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="26" t="n">
         <v>45304</v>
       </c>
-      <c r="C14" s="9" t="n">
-        <v>9267</v>
-      </c>
-      <c r="D14" s="9" t="n">
-        <v>8217</v>
+      <c r="C14" s="27" t="n">
+        <v>10696</v>
+      </c>
+      <c r="D14" s="27" t="n">
+        <v>4225</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>189</v>
-      </c>
-      <c r="F14" s="10" t="n">
-        <v>77.04000000000001</v>
+        <v>100</v>
+      </c>
+      <c r="F14" s="28" t="n">
+        <v>55.41</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="4" t="n">
+      <c r="B15" s="23" t="n">
         <v>45305</v>
       </c>
-      <c r="C15" s="5" t="n">
-        <v>7667</v>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>4666</v>
+      <c r="C15" s="24" t="n">
+        <v>10824</v>
+      </c>
+      <c r="D15" s="24" t="n">
+        <v>8800</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>142</v>
-      </c>
-      <c r="F15" s="6" t="n">
-        <v>82.67</v>
+        <v>109</v>
+      </c>
+      <c r="F15" s="25" t="n">
+        <v>64.18000000000001</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="B16" s="8" t="n">
+      <c r="B16" s="26" t="n">
         <v>45306</v>
       </c>
-      <c r="C16" s="9" t="n">
-        <v>3912</v>
-      </c>
-      <c r="D16" s="9" t="n">
-        <v>5170</v>
+      <c r="C16" s="27" t="n">
+        <v>3471</v>
+      </c>
+      <c r="D16" s="27" t="n">
+        <v>8640</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>132</v>
-      </c>
-      <c r="F16" s="10" t="n">
-        <v>93.52</v>
+        <v>148</v>
+      </c>
+      <c r="F16" s="28" t="n">
+        <v>30.39</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="4" t="n">
+      <c r="B17" s="23" t="n">
         <v>45307</v>
       </c>
-      <c r="C17" s="5" t="n">
-        <v>8037</v>
-      </c>
-      <c r="D17" s="5" t="n">
-        <v>3453</v>
+      <c r="C17" s="24" t="n">
+        <v>10016</v>
+      </c>
+      <c r="D17" s="24" t="n">
+        <v>5289</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>96</v>
-      </c>
-      <c r="F17" s="6" t="n">
-        <v>63.69</v>
+        <v>135</v>
+      </c>
+      <c r="F17" s="25" t="n">
+        <v>116.82</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="8" t="n">
+      <c r="B18" s="26" t="n">
         <v>45308</v>
       </c>
-      <c r="C18" s="9" t="n">
-        <v>6656</v>
-      </c>
-      <c r="D18" s="9" t="n">
-        <v>4707</v>
+      <c r="C18" s="27" t="n">
+        <v>4800</v>
+      </c>
+      <c r="D18" s="27" t="n">
+        <v>2907</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>75</v>
-      </c>
-      <c r="F18" s="10" t="n">
-        <v>36.43</v>
+        <v>103</v>
+      </c>
+      <c r="F18" s="28" t="n">
+        <v>101.05</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B19" s="4" t="n">
+      <c r="B19" s="23" t="n">
         <v>45309</v>
       </c>
-      <c r="C19" s="5" t="n">
-        <v>3460</v>
-      </c>
-      <c r="D19" s="5" t="n">
-        <v>3627</v>
+      <c r="C19" s="24" t="n">
+        <v>8908</v>
+      </c>
+      <c r="D19" s="24" t="n">
+        <v>5464</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>170</v>
-      </c>
-      <c r="F19" s="6" t="n">
-        <v>72.2</v>
+        <v>166</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>96.87</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="8" t="n">
+      <c r="B20" s="26" t="n">
         <v>45310</v>
       </c>
-      <c r="C20" s="9" t="n">
-        <v>3444</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>5913</v>
+      <c r="C20" s="27" t="n">
+        <v>11640</v>
+      </c>
+      <c r="D20" s="27" t="n">
+        <v>9257</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>166</v>
-      </c>
-      <c r="F20" s="10" t="n">
-        <v>91.44</v>
+        <v>164</v>
+      </c>
+      <c r="F20" s="28" t="n">
+        <v>107.45</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B21" s="4" t="n">
+      <c r="B21" s="23" t="n">
         <v>45311</v>
       </c>
-      <c r="C21" s="5" t="n">
-        <v>3967</v>
-      </c>
-      <c r="D21" s="5" t="n">
-        <v>5077</v>
+      <c r="C21" s="24" t="n">
+        <v>5550</v>
+      </c>
+      <c r="D21" s="24" t="n">
+        <v>5100</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>63</v>
-      </c>
-      <c r="F21" s="6" t="n">
-        <v>39.06</v>
+        <v>162</v>
+      </c>
+      <c r="F21" s="25" t="n">
+        <v>30.33</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="8" t="n">
+      <c r="B22" s="26" t="n">
         <v>45312</v>
       </c>
-      <c r="C22" s="9" t="n">
-        <v>4991</v>
-      </c>
-      <c r="D22" s="9" t="n">
-        <v>6514</v>
+      <c r="C22" s="27" t="n">
+        <v>8127</v>
+      </c>
+      <c r="D22" s="27" t="n">
+        <v>10936</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>52</v>
-      </c>
-      <c r="F22" s="10" t="n">
-        <v>63.35</v>
+        <v>60</v>
+      </c>
+      <c r="F22" s="28" t="n">
+        <v>76.98999999999999</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="B23" s="4" t="n">
+      <c r="B23" s="23" t="n">
         <v>45313</v>
       </c>
-      <c r="C23" s="5" t="n">
-        <v>5105</v>
-      </c>
-      <c r="D23" s="5" t="n">
-        <v>8007</v>
+      <c r="C23" s="24" t="n">
+        <v>8358</v>
+      </c>
+      <c r="D23" s="24" t="n">
+        <v>8620</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>68</v>
-      </c>
-      <c r="F23" s="6" t="n">
-        <v>68.64</v>
+        <v>190</v>
+      </c>
+      <c r="F23" s="25" t="n">
+        <v>100.64</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
         <v>22</v>
       </c>
-      <c r="B24" s="8" t="n">
+      <c r="B24" s="26" t="n">
         <v>45314</v>
       </c>
-      <c r="C24" s="9" t="n">
-        <v>7339</v>
-      </c>
-      <c r="D24" s="9" t="n">
-        <v>5788</v>
+      <c r="C24" s="27" t="n">
+        <v>5483</v>
+      </c>
+      <c r="D24" s="27" t="n">
+        <v>4070</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>79</v>
-      </c>
-      <c r="F24" s="10" t="n">
-        <v>92.61</v>
+        <v>112</v>
+      </c>
+      <c r="F24" s="28" t="n">
+        <v>53.75</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="B25" s="4" t="n">
+      <c r="B25" s="23" t="n">
         <v>45315</v>
       </c>
-      <c r="C25" s="5" t="n">
-        <v>8131</v>
-      </c>
-      <c r="D25" s="5" t="n">
-        <v>4132</v>
+      <c r="C25" s="24" t="n">
+        <v>7200</v>
+      </c>
+      <c r="D25" s="24" t="n">
+        <v>7796</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>200</v>
-      </c>
-      <c r="F25" s="6" t="n">
-        <v>90.23999999999999</v>
+        <v>179</v>
+      </c>
+      <c r="F25" s="25" t="n">
+        <v>80.43000000000001</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="B26" s="8" t="n">
+      <c r="B26" s="26" t="n">
         <v>45316</v>
       </c>
-      <c r="C26" s="9" t="n">
-        <v>3417</v>
-      </c>
-      <c r="D26" s="9" t="n">
-        <v>5832</v>
+      <c r="C26" s="27" t="n">
+        <v>9560</v>
+      </c>
+      <c r="D26" s="27" t="n">
+        <v>9801</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>80</v>
-      </c>
-      <c r="F26" s="10" t="n">
-        <v>78.59999999999999</v>
+        <v>111</v>
+      </c>
+      <c r="F26" s="28" t="n">
+        <v>96.53</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B27" s="4" t="n">
+      <c r="B27" s="23" t="n">
         <v>45317</v>
       </c>
-      <c r="C27" s="5" t="n">
-        <v>7797</v>
-      </c>
-      <c r="D27" s="5" t="n">
-        <v>5710</v>
+      <c r="C27" s="24" t="n">
+        <v>4932</v>
+      </c>
+      <c r="D27" s="24" t="n">
+        <v>6300</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>148</v>
-      </c>
-      <c r="F27" s="6" t="n">
-        <v>74.22</v>
+        <v>138</v>
+      </c>
+      <c r="F27" s="25" t="n">
+        <v>36.8</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
         <v>26</v>
       </c>
-      <c r="B28" s="8" t="n">
+      <c r="B28" s="26" t="n">
         <v>45318</v>
       </c>
-      <c r="C28" s="9" t="n">
-        <v>4828</v>
-      </c>
-      <c r="D28" s="9" t="n">
-        <v>4516</v>
+      <c r="C28" s="27" t="n">
+        <v>11288</v>
+      </c>
+      <c r="D28" s="27" t="n">
+        <v>4145</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>192</v>
-      </c>
-      <c r="F28" s="10" t="n">
-        <v>75.77</v>
+        <v>74</v>
+      </c>
+      <c r="F28" s="28" t="n">
+        <v>67.51000000000001</v>
       </c>
       <c r="G28" s="7" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B29" s="4" t="n">
+      <c r="B29" s="23" t="n">
         <v>45319</v>
       </c>
-      <c r="C29" s="5" t="n">
-        <v>9065</v>
-      </c>
-      <c r="D29" s="5" t="n">
-        <v>8290</v>
+      <c r="C29" s="24" t="n">
+        <v>7551</v>
+      </c>
+      <c r="D29" s="24" t="n">
+        <v>11824</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>56</v>
-      </c>
-      <c r="F29" s="6" t="n">
-        <v>54.73</v>
+        <v>135</v>
+      </c>
+      <c r="F29" s="25" t="n">
+        <v>47.46</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="B30" s="8" t="n">
+      <c r="B30" s="26" t="n">
         <v>45320</v>
       </c>
-      <c r="C30" s="9" t="n">
-        <v>8523</v>
-      </c>
-      <c r="D30" s="9" t="n">
-        <v>4987</v>
+      <c r="C30" s="27" t="n">
+        <v>3359</v>
+      </c>
+      <c r="D30" s="27" t="n">
+        <v>4464</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>138</v>
-      </c>
-      <c r="F30" s="10" t="n">
-        <v>73</v>
+        <v>161</v>
+      </c>
+      <c r="F30" s="28" t="n">
+        <v>65.86</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="B31" s="4" t="n">
+      <c r="B31" s="23" t="n">
         <v>45321</v>
       </c>
-      <c r="C31" s="5" t="n">
-        <v>8945</v>
-      </c>
-      <c r="D31" s="5" t="n">
-        <v>8549</v>
+      <c r="C31" s="24" t="n">
+        <v>4800</v>
+      </c>
+      <c r="D31" s="24" t="n">
+        <v>11962</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>137</v>
-      </c>
-      <c r="F31" s="6" t="n">
-        <v>53.02</v>
+        <v>127</v>
+      </c>
+      <c r="F31" s="25" t="n">
+        <v>71.47</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="B32" s="8" t="n">
+      <c r="B32" s="26" t="n">
         <v>45322</v>
       </c>
-      <c r="C32" s="9" t="n">
-        <v>7664</v>
-      </c>
-      <c r="D32" s="9" t="n">
-        <v>8399</v>
+      <c r="C32" s="27" t="n">
+        <v>3438</v>
+      </c>
+      <c r="D32" s="27" t="n">
+        <v>8689</v>
       </c>
       <c r="E32" s="7" t="n">
-        <v>192</v>
-      </c>
-      <c r="F32" s="10" t="n">
-        <v>88.27</v>
+        <v>93</v>
+      </c>
+      <c r="F32" s="28" t="n">
+        <v>111.16</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>12</v>
@@ -1304,411 +1325,411 @@
       <c r="A33" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="B33" s="4" t="n">
+      <c r="B33" s="23" t="n">
         <v>45323</v>
       </c>
-      <c r="C33" s="5" t="n">
-        <v>6636</v>
-      </c>
-      <c r="D33" s="5" t="n">
-        <v>8108</v>
+      <c r="C33" s="24" t="n">
+        <v>9684</v>
+      </c>
+      <c r="D33" s="24" t="n">
+        <v>8800</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>159</v>
-      </c>
-      <c r="F33" s="6" t="n">
-        <v>58.25</v>
+        <v>167</v>
+      </c>
+      <c r="F33" s="25" t="n">
+        <v>80.56999999999999</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
         <v>32</v>
       </c>
-      <c r="B34" s="8" t="n">
+      <c r="B34" s="26" t="n">
         <v>45324</v>
       </c>
-      <c r="C34" s="9" t="n">
-        <v>5005</v>
-      </c>
-      <c r="D34" s="9" t="n">
-        <v>3384</v>
+      <c r="C34" s="27" t="n">
+        <v>7183</v>
+      </c>
+      <c r="D34" s="27" t="n">
+        <v>3580</v>
       </c>
       <c r="E34" s="7" t="n">
-        <v>175</v>
-      </c>
-      <c r="F34" s="10" t="n">
-        <v>44.61</v>
+        <v>152</v>
+      </c>
+      <c r="F34" s="28" t="n">
+        <v>52.52</v>
       </c>
       <c r="G34" s="7" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="B35" s="4" t="n">
+      <c r="B35" s="23" t="n">
         <v>45325</v>
       </c>
-      <c r="C35" s="5" t="n">
-        <v>6879</v>
-      </c>
-      <c r="D35" s="5" t="n">
-        <v>7790</v>
+      <c r="C35" s="24" t="n">
+        <v>8596</v>
+      </c>
+      <c r="D35" s="24" t="n">
+        <v>3945</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>104</v>
-      </c>
-      <c r="F35" s="6" t="n">
-        <v>32.29</v>
+        <v>178</v>
+      </c>
+      <c r="F35" s="25" t="n">
+        <v>81.54000000000001</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
         <v>34</v>
       </c>
-      <c r="B36" s="8" t="n">
+      <c r="B36" s="26" t="n">
         <v>45326</v>
       </c>
-      <c r="C36" s="9" t="n">
-        <v>8027</v>
-      </c>
-      <c r="D36" s="9" t="n">
-        <v>8001</v>
+      <c r="C36" s="27" t="n">
+        <v>9500</v>
+      </c>
+      <c r="D36" s="27" t="n">
+        <v>4353</v>
       </c>
       <c r="E36" s="7" t="n">
-        <v>181</v>
-      </c>
-      <c r="F36" s="10" t="n">
-        <v>29.41</v>
+        <v>107</v>
+      </c>
+      <c r="F36" s="28" t="n">
+        <v>104.4</v>
       </c>
       <c r="G36" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="B37" s="4" t="n">
+      <c r="B37" s="23" t="n">
         <v>45327</v>
       </c>
-      <c r="C37" s="5" t="n">
-        <v>5478</v>
-      </c>
-      <c r="D37" s="5" t="n">
-        <v>4201</v>
+      <c r="C37" s="24" t="n">
+        <v>6413</v>
+      </c>
+      <c r="D37" s="24" t="n">
+        <v>6849</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>42</v>
-      </c>
-      <c r="F37" s="6" t="n">
-        <v>65.11</v>
+        <v>181</v>
+      </c>
+      <c r="F37" s="25" t="n">
+        <v>89.84999999999999</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n">
         <v>36</v>
       </c>
-      <c r="B38" s="8" t="n">
+      <c r="B38" s="26" t="n">
         <v>45328</v>
       </c>
-      <c r="C38" s="9" t="n">
-        <v>3253</v>
-      </c>
-      <c r="D38" s="9" t="n">
-        <v>7175</v>
+      <c r="C38" s="27" t="n">
+        <v>11141</v>
+      </c>
+      <c r="D38" s="27" t="n">
+        <v>5100</v>
       </c>
       <c r="E38" s="7" t="n">
-        <v>69</v>
-      </c>
-      <c r="F38" s="10" t="n">
-        <v>67.43000000000001</v>
+        <v>196</v>
+      </c>
+      <c r="F38" s="28" t="n">
+        <v>51.56</v>
       </c>
       <c r="G38" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="B39" s="4" t="n">
+      <c r="B39" s="23" t="n">
         <v>45329</v>
       </c>
-      <c r="C39" s="5" t="n">
-        <v>9416</v>
-      </c>
-      <c r="D39" s="5" t="n">
-        <v>4805</v>
+      <c r="C39" s="24" t="n">
+        <v>2124</v>
+      </c>
+      <c r="D39" s="24" t="n">
+        <v>4910</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>177</v>
-      </c>
-      <c r="F39" s="6" t="n">
-        <v>28.48</v>
+        <v>193</v>
+      </c>
+      <c r="F39" s="25" t="n">
+        <v>31.39</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="n">
         <v>38</v>
       </c>
-      <c r="B40" s="8" t="n">
+      <c r="B40" s="26" t="n">
         <v>45330</v>
       </c>
-      <c r="C40" s="9" t="n">
-        <v>4507</v>
-      </c>
-      <c r="D40" s="9" t="n">
-        <v>4138</v>
+      <c r="C40" s="27" t="n">
+        <v>8966</v>
+      </c>
+      <c r="D40" s="27" t="n">
+        <v>8715</v>
       </c>
       <c r="E40" s="7" t="n">
-        <v>108</v>
-      </c>
-      <c r="F40" s="10" t="n">
-        <v>75.43000000000001</v>
+        <v>186</v>
+      </c>
+      <c r="F40" s="28" t="n">
+        <v>36.49</v>
       </c>
       <c r="G40" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
         <v>39</v>
       </c>
-      <c r="B41" s="4" t="n">
+      <c r="B41" s="23" t="n">
         <v>45331</v>
       </c>
-      <c r="C41" s="5" t="n">
-        <v>8919</v>
-      </c>
-      <c r="D41" s="5" t="n">
-        <v>6586</v>
+      <c r="C41" s="24" t="n">
+        <v>5338</v>
+      </c>
+      <c r="D41" s="24" t="n">
+        <v>4384</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>127</v>
-      </c>
-      <c r="F41" s="6" t="n">
-        <v>31.94</v>
+        <v>196</v>
+      </c>
+      <c r="F41" s="25" t="n">
+        <v>54.78</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="B42" s="8" t="n">
+      <c r="B42" s="26" t="n">
         <v>45332</v>
       </c>
-      <c r="C42" s="9" t="n">
-        <v>6662</v>
-      </c>
-      <c r="D42" s="9" t="n">
-        <v>5908</v>
+      <c r="C42" s="27" t="n">
+        <v>7939</v>
+      </c>
+      <c r="D42" s="27" t="n">
+        <v>5400</v>
       </c>
       <c r="E42" s="7" t="n">
-        <v>68</v>
-      </c>
-      <c r="F42" s="10" t="n">
-        <v>32.52</v>
+        <v>141</v>
+      </c>
+      <c r="F42" s="28" t="n">
+        <v>67.25</v>
       </c>
       <c r="G42" s="7" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n">
         <v>41</v>
       </c>
-      <c r="B43" s="4" t="n">
+      <c r="B43" s="23" t="n">
         <v>45333</v>
       </c>
-      <c r="C43" s="5" t="n">
-        <v>5987</v>
-      </c>
-      <c r="D43" s="5" t="n">
-        <v>5011</v>
+      <c r="C43" s="24" t="n">
+        <v>10754</v>
+      </c>
+      <c r="D43" s="24" t="n">
+        <v>11190</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>115</v>
-      </c>
-      <c r="F43" s="6" t="n">
-        <v>30.1</v>
+        <v>94</v>
+      </c>
+      <c r="F43" s="25" t="n">
+        <v>82.93000000000001</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
         <v>42</v>
       </c>
-      <c r="B44" s="8" t="n">
+      <c r="B44" s="26" t="n">
         <v>45334</v>
       </c>
-      <c r="C44" s="9" t="n">
-        <v>5476</v>
-      </c>
-      <c r="D44" s="9" t="n">
-        <v>8042</v>
+      <c r="C44" s="27" t="n">
+        <v>7200</v>
+      </c>
+      <c r="D44" s="27" t="n">
+        <v>7228</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>151</v>
-      </c>
-      <c r="F44" s="10" t="n">
-        <v>50.14</v>
+        <v>161</v>
+      </c>
+      <c r="F44" s="28" t="n">
+        <v>33.25</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n">
         <v>43</v>
       </c>
-      <c r="B45" s="4" t="n">
+      <c r="B45" s="23" t="n">
         <v>45335</v>
       </c>
-      <c r="C45" s="5" t="n">
-        <v>4473</v>
-      </c>
-      <c r="D45" s="5" t="n">
-        <v>8437</v>
+      <c r="C45" s="24" t="n">
+        <v>9570</v>
+      </c>
+      <c r="D45" s="24" t="n">
+        <v>10177</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>80</v>
-      </c>
-      <c r="F45" s="6" t="n">
-        <v>62.45</v>
+        <v>190</v>
+      </c>
+      <c r="F45" s="25" t="n">
+        <v>50.7</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n">
         <v>44</v>
       </c>
-      <c r="B46" s="8" t="n">
+      <c r="B46" s="26" t="n">
         <v>45336</v>
       </c>
-      <c r="C46" s="9" t="n">
-        <v>4963</v>
-      </c>
-      <c r="D46" s="9" t="n">
-        <v>7362</v>
+      <c r="C46" s="27" t="n">
+        <v>10497</v>
+      </c>
+      <c r="D46" s="27" t="n">
+        <v>5832</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>156</v>
-      </c>
-      <c r="F46" s="10" t="n">
-        <v>46.66</v>
+        <v>100</v>
+      </c>
+      <c r="F46" s="28" t="n">
+        <v>105.41</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n">
         <v>45</v>
       </c>
-      <c r="B47" s="4" t="n">
+      <c r="B47" s="23" t="n">
         <v>45337</v>
       </c>
-      <c r="C47" s="5" t="n">
-        <v>9454</v>
-      </c>
-      <c r="D47" s="5" t="n">
-        <v>4599</v>
+      <c r="C47" s="24" t="n">
+        <v>5245</v>
+      </c>
+      <c r="D47" s="24" t="n">
+        <v>6220</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="F47" s="6" t="n">
-        <v>60.52</v>
+        <v>166</v>
+      </c>
+      <c r="F47" s="25" t="n">
+        <v>50.66</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n">
         <v>46</v>
       </c>
-      <c r="B48" s="8" t="n">
+      <c r="B48" s="26" t="n">
         <v>45338</v>
       </c>
-      <c r="C48" s="9" t="n">
-        <v>5957</v>
-      </c>
-      <c r="D48" s="9" t="n">
-        <v>8408</v>
+      <c r="C48" s="27" t="n">
+        <v>11920</v>
+      </c>
+      <c r="D48" s="27" t="n">
+        <v>3920</v>
       </c>
       <c r="E48" s="7" t="n">
-        <v>107</v>
-      </c>
-      <c r="F48" s="10" t="n">
-        <v>64.13</v>
+        <v>89</v>
+      </c>
+      <c r="F48" s="28" t="n">
+        <v>73.62</v>
       </c>
       <c r="G48" s="7" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
         <v>47</v>
       </c>
-      <c r="B49" s="4" t="n">
+      <c r="B49" s="23" t="n">
         <v>45339</v>
       </c>
-      <c r="C49" s="5" t="n">
-        <v>4037</v>
-      </c>
-      <c r="D49" s="5" t="n">
-        <v>5456</v>
+      <c r="C49" s="24" t="n">
+        <v>9580</v>
+      </c>
+      <c r="D49" s="24" t="n">
+        <v>7926</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>168</v>
-      </c>
-      <c r="F49" s="6" t="n">
-        <v>76.45999999999999</v>
+        <v>130</v>
+      </c>
+      <c r="F49" s="25" t="n">
+        <v>89.12</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="n">
         <v>48</v>
       </c>
-      <c r="B50" s="8" t="n">
+      <c r="B50" s="26" t="n">
         <v>45340</v>
       </c>
-      <c r="C50" s="9" t="n">
-        <v>3959</v>
-      </c>
-      <c r="D50" s="9" t="n">
-        <v>3258</v>
+      <c r="C50" s="27" t="n">
+        <v>2840</v>
+      </c>
+      <c r="D50" s="27" t="n">
+        <v>5046</v>
       </c>
       <c r="E50" s="7" t="n">
-        <v>85</v>
-      </c>
-      <c r="F50" s="10" t="n">
-        <v>87.12</v>
+        <v>110</v>
+      </c>
+      <c r="F50" s="28" t="n">
+        <v>99.8</v>
       </c>
       <c r="G50" s="7" t="n">
         <v>5</v>
@@ -1718,181 +1739,181 @@
       <c r="A51" s="3" t="n">
         <v>49</v>
       </c>
-      <c r="B51" s="4" t="n">
+      <c r="B51" s="23" t="n">
         <v>45341</v>
       </c>
-      <c r="C51" s="5" t="n">
-        <v>6312</v>
-      </c>
-      <c r="D51" s="5" t="n">
-        <v>4676</v>
+      <c r="C51" s="24" t="n">
+        <v>7857</v>
+      </c>
+      <c r="D51" s="24" t="n">
+        <v>6300</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>169</v>
-      </c>
-      <c r="F51" s="6" t="n">
-        <v>66.61</v>
+        <v>150</v>
+      </c>
+      <c r="F51" s="25" t="n">
+        <v>88.73</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="B52" s="8" t="n">
+      <c r="B52" s="26" t="n">
         <v>45342</v>
       </c>
-      <c r="C52" s="9" t="n">
-        <v>3992</v>
-      </c>
-      <c r="D52" s="9" t="n">
-        <v>3062</v>
+      <c r="C52" s="27" t="n">
+        <v>4115</v>
+      </c>
+      <c r="D52" s="27" t="n">
+        <v>10212</v>
       </c>
       <c r="E52" s="7" t="n">
-        <v>67</v>
-      </c>
-      <c r="F52" s="10" t="n">
-        <v>44.28</v>
+        <v>89</v>
+      </c>
+      <c r="F52" s="28" t="n">
+        <v>95.23</v>
       </c>
       <c r="G52" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n">
         <v>51</v>
       </c>
-      <c r="B53" s="4" t="n">
+      <c r="B53" s="23" t="n">
         <v>45343</v>
       </c>
-      <c r="C53" s="5" t="n">
-        <v>6140</v>
-      </c>
-      <c r="D53" s="5" t="n">
-        <v>5384</v>
+      <c r="C53" s="24" t="n">
+        <v>5536</v>
+      </c>
+      <c r="D53" s="24" t="n">
+        <v>6713</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>200</v>
-      </c>
-      <c r="F53" s="6" t="n">
-        <v>59.69</v>
+        <v>98</v>
+      </c>
+      <c r="F53" s="25" t="n">
+        <v>79.08</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="n">
         <v>52</v>
       </c>
-      <c r="B54" s="8" t="n">
+      <c r="B54" s="26" t="n">
         <v>45344</v>
       </c>
-      <c r="C54" s="9" t="n">
-        <v>6017</v>
-      </c>
-      <c r="D54" s="9" t="n">
-        <v>6086</v>
+      <c r="C54" s="27" t="n">
+        <v>4634</v>
+      </c>
+      <c r="D54" s="27" t="n">
+        <v>2182</v>
       </c>
       <c r="E54" s="7" t="n">
-        <v>116</v>
-      </c>
-      <c r="F54" s="10" t="n">
-        <v>55.27</v>
+        <v>191</v>
+      </c>
+      <c r="F54" s="28" t="n">
+        <v>88.2</v>
       </c>
       <c r="G54" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n">
         <v>53</v>
       </c>
-      <c r="B55" s="4" t="n">
+      <c r="B55" s="23" t="n">
         <v>45345</v>
       </c>
-      <c r="C55" s="5" t="n">
-        <v>8145</v>
-      </c>
-      <c r="D55" s="5" t="n">
-        <v>4993</v>
+      <c r="C55" s="24" t="n">
+        <v>9237</v>
+      </c>
+      <c r="D55" s="24" t="n">
+        <v>8800</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>169</v>
-      </c>
-      <c r="F55" s="6" t="n">
-        <v>34.32</v>
+        <v>150</v>
+      </c>
+      <c r="F55" s="25" t="n">
+        <v>108.38</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="n">
         <v>54</v>
       </c>
-      <c r="B56" s="8" t="n">
+      <c r="B56" s="26" t="n">
         <v>45346</v>
       </c>
-      <c r="C56" s="9" t="n">
-        <v>5366</v>
-      </c>
-      <c r="D56" s="9" t="n">
-        <v>3342</v>
+      <c r="C56" s="27" t="n">
+        <v>11755</v>
+      </c>
+      <c r="D56" s="27" t="n">
+        <v>2781</v>
       </c>
       <c r="E56" s="7" t="n">
-        <v>195</v>
-      </c>
-      <c r="F56" s="10" t="n">
-        <v>72.15000000000001</v>
+        <v>101</v>
+      </c>
+      <c r="F56" s="28" t="n">
+        <v>60.61</v>
       </c>
       <c r="G56" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n">
         <v>55</v>
       </c>
-      <c r="B57" s="4" t="n">
+      <c r="B57" s="23" t="n">
         <v>45347</v>
       </c>
-      <c r="C57" s="5" t="n">
-        <v>3555</v>
-      </c>
-      <c r="D57" s="5" t="n">
-        <v>4528</v>
+      <c r="C57" s="24" t="n">
+        <v>4910</v>
+      </c>
+      <c r="D57" s="24" t="n">
+        <v>7528</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>90</v>
-      </c>
-      <c r="F57" s="6" t="n">
-        <v>51.74</v>
+        <v>147</v>
+      </c>
+      <c r="F57" s="25" t="n">
+        <v>102.85</v>
       </c>
       <c r="G57" s="3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="n">
         <v>56</v>
       </c>
-      <c r="B58" s="8" t="n">
+      <c r="B58" s="26" t="n">
         <v>45348</v>
       </c>
-      <c r="C58" s="9" t="n">
-        <v>9177</v>
-      </c>
-      <c r="D58" s="9" t="n">
-        <v>7446</v>
+      <c r="C58" s="27" t="n">
+        <v>9500</v>
+      </c>
+      <c r="D58" s="27" t="n">
+        <v>5544</v>
       </c>
       <c r="E58" s="7" t="n">
-        <v>79</v>
-      </c>
-      <c r="F58" s="10" t="n">
-        <v>55.54</v>
+        <v>108</v>
+      </c>
+      <c r="F58" s="28" t="n">
+        <v>57.67</v>
       </c>
       <c r="G58" s="7" t="n">
         <v>3</v>
@@ -1902,66 +1923,66 @@
       <c r="A59" s="3" t="n">
         <v>57</v>
       </c>
-      <c r="B59" s="4" t="n">
+      <c r="B59" s="23" t="n">
         <v>45349</v>
       </c>
-      <c r="C59" s="5" t="n">
-        <v>6963</v>
-      </c>
-      <c r="D59" s="5" t="n">
-        <v>5377</v>
+      <c r="C59" s="24" t="n">
+        <v>4883</v>
+      </c>
+      <c r="D59" s="24" t="n">
+        <v>8176</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>135</v>
-      </c>
-      <c r="F59" s="6" t="n">
-        <v>85.88</v>
+        <v>97</v>
+      </c>
+      <c r="F59" s="25" t="n">
+        <v>74.69</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="n">
         <v>58</v>
       </c>
-      <c r="B60" s="8" t="n">
+      <c r="B60" s="26" t="n">
         <v>45350</v>
       </c>
-      <c r="C60" s="9" t="n">
-        <v>7592</v>
-      </c>
-      <c r="D60" s="9" t="n">
-        <v>4541</v>
+      <c r="C60" s="27" t="n">
+        <v>2607</v>
+      </c>
+      <c r="D60" s="27" t="n">
+        <v>8538</v>
       </c>
       <c r="E60" s="7" t="n">
-        <v>81</v>
-      </c>
-      <c r="F60" s="10" t="n">
-        <v>31.63</v>
+        <v>119</v>
+      </c>
+      <c r="F60" s="28" t="n">
+        <v>63.92</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n">
         <v>59</v>
       </c>
-      <c r="B61" s="4" t="n">
+      <c r="B61" s="23" t="n">
         <v>45351</v>
       </c>
-      <c r="C61" s="5" t="n">
-        <v>4222</v>
-      </c>
-      <c r="D61" s="5" t="n">
-        <v>8169</v>
+      <c r="C61" s="24" t="n">
+        <v>3798</v>
+      </c>
+      <c r="D61" s="24" t="n">
+        <v>7517</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>178</v>
-      </c>
-      <c r="F61" s="6" t="n">
-        <v>71.78</v>
+        <v>120</v>
+      </c>
+      <c r="F61" s="25" t="n">
+        <v>81.01000000000001</v>
       </c>
       <c r="G61" s="3" t="n">
         <v>2</v>
@@ -1971,23 +1992,23 @@
       <c r="A62" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="B62" s="8" t="n">
+      <c r="B62" s="26" t="n">
         <v>45352</v>
       </c>
-      <c r="C62" s="9" t="n">
-        <v>6300</v>
-      </c>
-      <c r="D62" s="9" t="n">
-        <v>6889</v>
+      <c r="C62" s="27" t="n">
+        <v>2381</v>
+      </c>
+      <c r="D62" s="27" t="n">
+        <v>8543</v>
       </c>
       <c r="E62" s="7" t="n">
-        <v>175</v>
-      </c>
-      <c r="F62" s="10" t="n">
-        <v>71.29000000000001</v>
+        <v>101</v>
+      </c>
+      <c r="F62" s="28" t="n">
+        <v>108.79</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -2068,11 +2089,11 @@
           <t>Minimum</t>
         </is>
       </c>
-      <c r="B4" s="15">
+      <c r="B4" s="29">
         <f>MIN(Sales_Data!C3:C62)</f>
         <v/>
       </c>
-      <c r="C4" s="15">
+      <c r="C4" s="29">
         <f>MIN(Sales_Data!D3:D62)</f>
         <v/>
       </c>
@@ -2088,11 +2109,11 @@
           <t>Maximum</t>
         </is>
       </c>
-      <c r="B5" s="15">
+      <c r="B5" s="29">
         <f>MAX(Sales_Data!C3:C62)</f>
         <v/>
       </c>
-      <c r="C5" s="15">
+      <c r="C5" s="29">
         <f>MAX(Sales_Data!D3:D62)</f>
         <v/>
       </c>
@@ -2108,11 +2129,11 @@
           <t>Range</t>
         </is>
       </c>
-      <c r="B6" s="15">
+      <c r="B6" s="29">
         <f>MAX(Sales_Data!C3:C62)-MIN(Sales_Data!C3:C62)</f>
         <v/>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="29">
         <f>MAX(Sales_Data!D3:D62)-MIN(Sales_Data!D3:D62)</f>
         <v/>
       </c>
@@ -2128,11 +2149,11 @@
           <t>Mean (Average)</t>
         </is>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="29">
         <f>AVERAGE(Sales_Data!C3:C62)</f>
         <v/>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="29">
         <f>AVERAGE(Sales_Data!D3:D62)</f>
         <v/>
       </c>
@@ -2168,17 +2189,17 @@
           <t>Mode</t>
         </is>
       </c>
-      <c r="B9" s="15">
-        <f>MODE(Sales_Data!C3:C62)</f>
-        <v/>
-      </c>
-      <c r="C9" s="15">
-        <f>MODE(Sales_Data!D3:D62)</f>
+      <c r="B9" s="29">
+        <f>IFERROR(MODE.SNGL(Sales_Data!C3:C62),"No mode")</f>
+        <v/>
+      </c>
+      <c r="C9" s="29">
+        <f>IFERROR(MODE.SNGL(Sales_Data!D3:D62),"No mode")</f>
         <v/>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Most frequently occurring value</t>
+          <t>Most frequently occurring value (IFERROR handles datasets with no repeats)</t>
         </is>
       </c>
     </row>
@@ -2188,11 +2209,11 @@
           <t>Variance (Sample)</t>
         </is>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="29">
         <f>VAR.S(Sales_Data!C3:C62)</f>
         <v/>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="29">
         <f>VAR.S(Sales_Data!D3:D62)</f>
         <v/>
       </c>
@@ -2208,11 +2229,11 @@
           <t>Std Dev (Sample)</t>
         </is>
       </c>
-      <c r="B11" s="15">
+      <c r="B11" s="29">
         <f>STDEV.S(Sales_Data!C3:C62)</f>
         <v/>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="29">
         <f>STDEV.S(Sales_Data!D3:D62)</f>
         <v/>
       </c>
@@ -2228,11 +2249,11 @@
           <t>Std Dev (Population)</t>
         </is>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="29">
         <f>STDEV.P(Sales_Data!C3:C62)</f>
         <v/>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="29">
         <f>STDEV.P(Sales_Data!D3:D62)</f>
         <v/>
       </c>
@@ -2288,11 +2309,11 @@
           <t>1st Quartile (Q1)</t>
         </is>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="29">
         <f>QUARTILE.INC(Sales_Data!C3:C62,1)</f>
         <v/>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="29">
         <f>QUARTILE.INC(Sales_Data!D3:D62,1)</f>
         <v/>
       </c>
@@ -2308,11 +2329,11 @@
           <t>3rd Quartile (Q3)</t>
         </is>
       </c>
-      <c r="B16" s="15">
+      <c r="B16" s="29">
         <f>QUARTILE.INC(Sales_Data!C3:C62,3)</f>
         <v/>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="29">
         <f>QUARTILE.INC(Sales_Data!D3:D62,3)</f>
         <v/>
       </c>
@@ -2328,11 +2349,11 @@
           <t>IQR (Q3 - Q1)</t>
         </is>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="29">
         <f>QUARTILE.INC(Sales_Data!C3:C62,3)-QUARTILE.INC(Sales_Data!C3:C62,1)</f>
         <v/>
       </c>
-      <c r="C17" s="15">
+      <c r="C17" s="29">
         <f>QUARTILE.INC(Sales_Data!D3:D62,3)-QUARTILE.INC(Sales_Data!D3:D62,1)</f>
         <v/>
       </c>
@@ -2348,11 +2369,11 @@
           <t>90th Percentile</t>
         </is>
       </c>
-      <c r="B18" s="15">
+      <c r="B18" s="29">
         <f>PERCENTILE.INC(Sales_Data!C3:C62,0.9)</f>
         <v/>
       </c>
-      <c r="C18" s="15">
+      <c r="C18" s="29">
         <f>PERCENTILE.INC(Sales_Data!D3:D62,0.9)</f>
         <v/>
       </c>
@@ -2388,11 +2409,11 @@
           <t>Standard Error</t>
         </is>
       </c>
-      <c r="B20" s="15">
+      <c r="B20" s="29">
         <f>STDEV.S(Sales_Data!C3:C62)/SQRT(COUNT(Sales_Data!C3:C62))</f>
         <v/>
       </c>
-      <c r="C20" s="15">
+      <c r="C20" s="29">
         <f>STDEV.S(Sales_Data!D3:D62)/SQRT(COUNT(Sales_Data!D3:D62))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Fix #NAME? errors: replace dot-notation functions with compatible equivalents in 02_Descriptive_Statistics.xlsx
</commit_message>
<xml_diff>
--- a/rFLA300/chapter-12/02_Descriptive_Statistics.xlsx
+++ b/rFLA300/chapter-12/02_Descriptive_Statistics.xlsx
@@ -2190,11 +2190,11 @@
         </is>
       </c>
       <c r="B9" s="29">
-        <f>IFERROR(MODE.SNGL(Sales_Data!C3:C62),"No mode")</f>
+        <f>IFERROR(MODE(Sales_Data!C3:C62),"No mode")</f>
         <v/>
       </c>
       <c r="C9" s="29">
-        <f>IFERROR(MODE.SNGL(Sales_Data!D3:D62),"No mode")</f>
+        <f>IFERROR(MODE(Sales_Data!D3:D62),"No mode")</f>
         <v/>
       </c>
       <c r="D9" s="13" t="inlineStr">
@@ -2210,11 +2210,11 @@
         </is>
       </c>
       <c r="B10" s="29">
-        <f>VAR.S(Sales_Data!C3:C62)</f>
+        <f>VAR(Sales_Data!C3:C62)</f>
         <v/>
       </c>
       <c r="C10" s="29">
-        <f>VAR.S(Sales_Data!D3:D62)</f>
+        <f>VAR(Sales_Data!D3:D62)</f>
         <v/>
       </c>
       <c r="D10" s="16" t="inlineStr">
@@ -2230,11 +2230,11 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>STDEV.S(Sales_Data!C3:C62)</f>
+        <f>STDEV(Sales_Data!C3:C62)</f>
         <v/>
       </c>
       <c r="C11" s="29">
-        <f>STDEV.S(Sales_Data!D3:D62)</f>
+        <f>STDEV(Sales_Data!D3:D62)</f>
         <v/>
       </c>
       <c r="D11" s="13" t="inlineStr">
@@ -2250,16 +2250,16 @@
         </is>
       </c>
       <c r="B12" s="29">
-        <f>STDEV.P(Sales_Data!C3:C62)</f>
+        <f>STDEVP(Sales_Data!C3:C62)</f>
         <v/>
       </c>
       <c r="C12" s="29">
-        <f>STDEV.P(Sales_Data!D3:D62)</f>
+        <f>STDEVP(Sales_Data!D3:D62)</f>
         <v/>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>Use when data IS the whole population</t>
+          <t>Use when data IS the whole population (STDEVP)</t>
         </is>
       </c>
     </row>
@@ -2310,11 +2310,11 @@
         </is>
       </c>
       <c r="B15" s="29">
-        <f>QUARTILE.INC(Sales_Data!C3:C62,1)</f>
+        <f>QUARTILE(Sales_Data!C3:C62,1)</f>
         <v/>
       </c>
       <c r="C15" s="29">
-        <f>QUARTILE.INC(Sales_Data!D3:D62,1)</f>
+        <f>QUARTILE(Sales_Data!D3:D62,1)</f>
         <v/>
       </c>
       <c r="D15" s="13" t="inlineStr">
@@ -2330,11 +2330,11 @@
         </is>
       </c>
       <c r="B16" s="29">
-        <f>QUARTILE.INC(Sales_Data!C3:C62,3)</f>
+        <f>QUARTILE(Sales_Data!C3:C62,3)</f>
         <v/>
       </c>
       <c r="C16" s="29">
-        <f>QUARTILE.INC(Sales_Data!D3:D62,3)</f>
+        <f>QUARTILE(Sales_Data!D3:D62,3)</f>
         <v/>
       </c>
       <c r="D16" s="16" t="inlineStr">
@@ -2350,11 +2350,11 @@
         </is>
       </c>
       <c r="B17" s="29">
-        <f>QUARTILE.INC(Sales_Data!C3:C62,3)-QUARTILE.INC(Sales_Data!C3:C62,1)</f>
+        <f>QUARTILE(Sales_Data!C3:C62,3)-QUARTILE(Sales_Data!C3:C62,1)</f>
         <v/>
       </c>
       <c r="C17" s="29">
-        <f>QUARTILE.INC(Sales_Data!D3:D62,3)-QUARTILE.INC(Sales_Data!D3:D62,1)</f>
+        <f>QUARTILE(Sales_Data!D3:D62,3)-QUARTILE(Sales_Data!D3:D62,1)</f>
         <v/>
       </c>
       <c r="D17" s="13" t="inlineStr">
@@ -2370,11 +2370,11 @@
         </is>
       </c>
       <c r="B18" s="29">
-        <f>PERCENTILE.INC(Sales_Data!C3:C62,0.9)</f>
+        <f>PERCENTILE(Sales_Data!C3:C62,0.9)</f>
         <v/>
       </c>
       <c r="C18" s="29">
-        <f>PERCENTILE.INC(Sales_Data!D3:D62,0.9)</f>
+        <f>PERCENTILE(Sales_Data!D3:D62,0.9)</f>
         <v/>
       </c>
       <c r="D18" s="16" t="inlineStr">
@@ -2390,11 +2390,11 @@
         </is>
       </c>
       <c r="B19" s="17">
-        <f>STDEV.S(Sales_Data!C3:C62)/AVERAGE(Sales_Data!C3:C62)</f>
+        <f>STDEV(Sales_Data!C3:C62)/AVERAGE(Sales_Data!C3:C62)</f>
         <v/>
       </c>
       <c r="C19" s="17">
-        <f>STDEV.S(Sales_Data!D3:D62)/AVERAGE(Sales_Data!D3:D62)</f>
+        <f>STDEV(Sales_Data!D3:D62)/AVERAGE(Sales_Data!D3:D62)</f>
         <v/>
       </c>
       <c r="D19" s="13" t="inlineStr">
@@ -2410,11 +2410,11 @@
         </is>
       </c>
       <c r="B20" s="29">
-        <f>STDEV.S(Sales_Data!C3:C62)/SQRT(COUNT(Sales_Data!C3:C62))</f>
+        <f>STDEV(Sales_Data!C3:C62)/SQRT(COUNT(Sales_Data!C3:C62))</f>
         <v/>
       </c>
       <c r="C20" s="29">
-        <f>STDEV.S(Sales_Data!D3:D62)/SQRT(COUNT(Sales_Data!D3:D62))</f>
+        <f>STDEV(Sales_Data!D3:D62)/SQRT(COUNT(Sales_Data!D3:D62))</f>
         <v/>
       </c>
       <c r="D20" s="16" t="inlineStr">
@@ -2423,6 +2423,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="18" t="inlineStr">
         <is>
@@ -2430,6 +2431,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="50" customHeight="1">
       <c r="A24" s="19" t="inlineStr">
         <is>
@@ -2468,6 +2470,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="80" customHeight="1">
       <c r="A3" s="20" t="inlineStr">
         <is>
@@ -2489,6 +2492,8 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
+    <row r="5"/>
     <row r="6" ht="80" customHeight="1">
       <c r="A6" s="20" t="inlineStr">
         <is>
@@ -2509,6 +2514,8 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
     <row r="9" ht="80" customHeight="1">
       <c r="A9" s="20" t="inlineStr">
         <is>
@@ -2529,6 +2536,8 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12" ht="80" customHeight="1">
       <c r="A12" s="20" t="inlineStr">
         <is>
@@ -2551,6 +2560,8 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
+    <row r="14"/>
     <row r="15" ht="80" customHeight="1">
       <c r="A15" s="20" t="inlineStr">
         <is>
@@ -2578,6 +2589,8 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18" ht="80" customHeight="1">
       <c r="A18" s="20" t="inlineStr">
         <is>

</xml_diff>